<commit_message>
Match form rows to the real drop-down values and tab convention
The Category drop-down offers six values: holdover not reflected, sector
classification incorrect, account size classification incorrect,
buying-center grouping wrong, salesforce data issue, other. The compound
categories drafted earlier were not among them, so rows now use only
valid values and carry the same list as data validation.

The tabs are per director, not per rep, so the Ary Tsotras tab is shared
with the rest of his team. Rationales are prefixed with the requester's
name to match the convention already in use there, and Status is left
blank to match the existing rows rather than the instruction sheet's
example.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ts2axbN7gkuKLHruvpVkR
</commit_message>
<xml_diff>
--- a/territory/F27-Feedback-Form-Rows.xlsx
+++ b/territory/F27-Feedback-Form-Rows.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Rows for Team Tab" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Rows for Ary Tsotras tab" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -476,8 +476,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="104" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="108" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -556,14 +556,10 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>1) Account is held to Feb 1, 2027 as an FAC holdover. 2) The opportunity on it is dead, with no live communication. 3) A Feb 1 holdover is retained only by moving the opportunity to QO before that date, and a dead cycle has no path there. 4) Named contact Joseph Sacri is known to the future owner from Joseph's previous organisation, so there is an existing relationship available to restart it now. Business impact: five months of a restartable relationship going cold before the account changes hands.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover. 2) The opportunity on it is dead, with no live communication. 3) A Feb 1 holdover is retained only by moving the opportunity to QO before that date, and a dead cycle has no path there. 4) Named contact Joseph Sacri is known to me from his previous organisation, so there is an existing relationship available to restart it now. Business impact: five months of a restartable relationship going cold before the account changes hands.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -598,14 +594,10 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account, so there is nothing to move to QO before Feb 1. 3) Open Opportunities Proposal+ reads 0 in the territory export. 4) Same APEX group as MaxLinear, which is also held and whose opportunity is closed lost, so the group is being held as a unit with nothing live in it. Business impact: the holdover cannot achieve its purpose and delays coverage by five months.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account, so there is nothing to move to QO before Feb 1. 3) Open Opportunities Proposal+ reads 0 in the territory export. 4) Same APEX group as MaxLinear, which is also held and whose opportunity is closed lost, so the group is held as a unit with nothing live in it. Business impact: the holdover cannot achieve its purpose and delays coverage by five months.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -640,14 +632,10 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>1) Held to Feb 1, 2027 as an FAC holdover. 2) The opportunity is closed lost, with no communication on the account. 3) A closed lost opportunity cannot reach QO by Feb 1, so the holdover condition cannot be satisfied. 4) Same APEX group as Exar Corporation, which has no opportunity at all. Business impact: an entire APEX group held for five months with no live cycle in it.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover. 2) The opportunity is closed lost, with no communication on the account. 3) A closed lost opportunity cannot reach QO by Feb 1, so the holdover condition cannot be satisfied. 4) Same APEX group as Exar Corporation, which has no opportunity at all. Business impact: an entire APEX group held for five months with no live cycle in it.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -677,34 +665,30 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Holdover not reflected/owner change required?</t>
+          <t>Holdover not reflected</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>1) Held to Feb 1, 2027 as an FAC holdover. 2) The opportunity has died. 3) Black Rock City LLC (001f300001v97AfAAI) is the same organisation in the same APEX group, also held to Feb 1 under the same owner, and is a duplicate record. 4) Requesting both records release together and that Black Rock City LLC merge into this one. Business impact: two records for one organisation both frozen until February on a dead cycle.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover. 2) The opportunity has died. 3) Black Rock City LLC (001f300001v97AfAAI) is the same organisation in the same APEX group, also held to Feb 1 under the same owner, and is a duplicate record. 4) Asking that both records release together and that Black Rock City LLC merge into this one. Business impact: two records for one organisation both frozen until February on a dead cycle.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Samba Tv, Inc.</t>
+          <t>Black Rock City LLC</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://infotech.lightning.force.com/lightning/r/Account/001f300001v8JfRAAU/view</t>
+          <t>https://infotech.lightning.force.com/lightning/r/Account/001f300001v97AfAAI/view</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Josh Scott</t>
+          <t>Andrew Bell</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -724,29 +708,25 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account, so nothing can reach QO before the date. 3) ITRG status is Winback, meaning a lapsed membership sits on the account. 4) Winback accounts are the highest-intent segment of the incoming book and are time-sensitive. Business impact: the single strongest re-entry point in the arriving territory sits idle until February.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover with no opportunity on the record. 2) Same organisation as Burning Man Project (001a700000LEgFFAA1), same APEX group, same current owner. 3) Black Rock City LLC is the operating entity behind the event and Burning Man Project is the nonprofit. 4) Asking for release alongside Burning Man Project and a merge into that record. Business impact: a duplicate record independently frozen until February.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Irhythm Technologies, Inc.</t>
+          <t>Samba Tv, Inc.</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://infotech.lightning.force.com/lightning/r/Account/00140000011lkU3AAI/view</t>
+          <t>https://infotech.lightning.force.com/lightning/r/Account/001f300001v8JfRAAU/view</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Cameron McLean</t>
+          <t>Josh Scott</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -766,29 +746,25 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account. 3) Open Opportunities Proposal+ reads 0 in the territory export. 4) With nothing to advance to QO, the holdover has no condition it can satisfy. Business impact: five months of lost coverage on a viable California account with no offsetting continuity benefit.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account, so nothing can reach QO before the date. 3) ITRG status is Winback, so a lapsed membership sits on the account. 4) Winbacks are the highest-intent accounts in the arriving book and are time-sensitive. Business impact: the strongest re-entry point in the territory sits idle until February.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Irhythm Technologies, Inc.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://infotech.lightning.force.com/lightning/r/Account/0013300001lNQtMAAW/view</t>
+          <t>https://infotech.lightning.force.com/lightning/r/Account/00140000011lkU3AAI/view</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Akshat Singh</t>
+          <t>Cameron McLean</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -803,34 +779,30 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Holdover not reflected/owner change required?</t>
+          <t>Holdover not reflected</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account. 3) Separately, the APEX group is ThoughtSpot, which acquired Mode Analytics. If that group carries larges, the account may belong in LE rather than SMB. 4) Raising both together so the group question is settled before the account is worked. Business impact: either five months of dead hold, or an account worked in the wrong segment.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account. 3) Open Opportunities Proposal+ reads 0 in the territory export. 4) With nothing to advance to QO, the holdover has no condition it can satisfy. Business impact: five months of lost coverage on a viable California account with no offsetting continuity benefit.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Black Rock City LLC</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://infotech.lightning.force.com/lightning/r/Account/001f300001v97AfAAI/view</t>
+          <t>https://infotech.lightning.force.com/lightning/r/Account/0013300001lNQtMAAW/view</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Andrew Bell</t>
+          <t>Akshat Singh</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -845,19 +817,15 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Holdover not reflected/owner change required?</t>
+          <t>Holdover not reflected</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>1) Held to Feb 1, 2027 as an FAC holdover with no opportunity on the record. 2) This is the same organisation as Burning Man Project (001a700000LEgFFAA1), in the same APEX group and under the same current owner. 3) Black Rock City LLC is the operating entity behind the event; Burning Man Project is the nonprofit. 4) Requesting release with Burning Man Project and a merge into that record. Business impact: a duplicate record independently frozen until February.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Held to Feb 1, 2027 as an FAC holdover. 2) There is no opportunity on the account. 3) Separate flag on the same record: the APEX group is ThoughtSpot, which acquired Mode Analytics. If that group carries larges the account may sit in LE rather than SMB. 4) Raising both together so the grouping is settled before the account is worked. Business impact: either five months of dead hold, or an account worked in the wrong segment.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -887,19 +855,15 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Holdover not reflected/owner change required?</t>
+          <t>Salesforce data issue</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>1) Vir Biotechnology appears twice in the proposed book under one APEX group. 2) Record 001f30000218CZkAAM (Viable, California) arrives August 24, 2026 under Christine McKay. 3) This record is held to Feb 1, 2027 under Eric Witmer. 4) The same company is therefore split across two arrival dates and two current owners because of a duplicate record. Business impact: half of one account is unworkable until February for no reason other than a data duplicate.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
+          <t>Sairam: 1) Vir Biotechnology appears twice in the proposed book under one APEX group. 2) Record 001f30000218CZkAAM (Viable, California) arrives August 24, 2026 under Christine McKay. 3) This record is held to Feb 1, 2027 under Eric Witmer. 4) One company is therefore split across two arrival dates and two current owners purely because of a duplicate record. Business impact: half an account unworkable until February for no reason other than a data duplicate.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -929,36 +893,37 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Holdover not reflected/owner change required?</t>
+          <t>Salesforce data issue</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>1) Enable appears twice in the proposed book under one APEX group. 2) Record 0014y00002rSxEyAAK (Viable, California) is held to Feb 1, 2027 under Abhishek Narayan. 3) This record arrives August 24, 2026 with no current owner recorded. 4) A third record, Enable Benefits (Ontario, Non-Viable), is also held to Feb 1. Business impact: one company split across two arrival dates by duplicate records, with part of it arriving unowned.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+          <t>Sairam: 1) Enable appears twice in the proposed book under one APEX group. 2) Record 0014y00002rSxEyAAK (Viable, California) is held to Feb 1, 2027 under Abhishek Narayan. 3) This record arrives August 24, 2026 with no current owner recorded. 4) A third record, Enable Benefits (Ontario, Non-Viable), is also held to Feb 1. Business impact: one company split across two arrival dates by duplicate records, with part of it arriving unowned.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Before pasting</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Yellow cells need an Opportunity Link pulled from SFDC. Rows marked "None." have no opportunity, which is the evidence itself, so leave that text in place. Category values must be re-picked from the tab drop-down after pasting, since pasted text can break the validation. Paste into your team tab, not this sheet.</t>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Paste into the Ary Tsotras tab, which is shared across his whole team, so the rationales are prefixed with your name to match Wil Pemberton's convention. Category values are the six from the tab's drop-down, so they will validate on paste. Yellow cells need an Opportunity Link from SFDC. Rows reading 'None.' have no opportunity at all, which is the evidence itself, so leave that text in place. Status is left blank, matching the existing rows in the tab.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B13:H13"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Holdover not reflected,Sector classification incorrect,Account size classification incorrect,Buying-center grouping wrong,Salesforce data issue,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>